<commit_message>
DDL: restore log_filters seeds in MWPV_DB_Create.sql; Add CategoryItem columns; add sql/MWPV_DB_Create_origional.sql; update docs/CategoryItem Layout-gadget.xlsx
</commit_message>
<xml_diff>
--- a/MWPV/docs/CategoryItem Layout-gadget.xlsx
+++ b/MWPV/docs/CategoryItem Layout-gadget.xlsx
@@ -1,22 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pgmrd\My Drive\MWPV\MWPV\docs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F34021A8-82C1-449C-98E5-2CF4AA1C13CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
     <sheet name="Fields" sheetId="2" r:id="rId2"/>
     <sheet name="Visibility" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="100">
   <si>
     <t>Category</t>
   </si>
@@ -205,13 +211,130 @@
   </si>
   <si>
     <t>Freeform notes</t>
+  </si>
+  <si>
+    <t>CategoryItem/CI_Name</t>
+  </si>
+  <si>
+    <t>Password Name</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Can not be modified</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>This is the email recorded for the web site</t>
+  </si>
+  <si>
+    <t>Needs to be added to Category Item Table</t>
+  </si>
+  <si>
+    <t>CateogyryItem/CI_Email</t>
+  </si>
+  <si>
+    <t>Needs to be added to Category Item Table
+Not needed for files/folders and applications</t>
+  </si>
+  <si>
+    <t>CategoryItem/CI_Description</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Description of this password entry</t>
+  </si>
+  <si>
+    <t>Needs to be added to Category Item Table
+Required for any website</t>
+  </si>
+  <si>
+    <t>*** Should we create one json/clob with this
+and the account number in?</t>
+  </si>
+  <si>
+    <t>CategoryItemSecurityQuestions/SecurityQuestion</t>
+  </si>
+  <si>
+    <t>CategoryItemSequerityQuestions/SecurityAnswer</t>
+  </si>
+  <si>
+    <t>*** Not defined yet. Is it needed</t>
+  </si>
+  <si>
+    <t>PasswordBox</t>
+  </si>
+  <si>
+    <t>Multiline/PasswordBox</t>
+  </si>
+  <si>
+    <t>Name of this Password entry(app name/web site 
+name/encryupte file or folder name)</t>
+  </si>
+  <si>
+    <t>*** Is this the user id login?</t>
+  </si>
+  <si>
+    <t>CategoryItemPasswordHistory/CIPaH_Password</t>
+  </si>
+  <si>
+    <t>Needs to be defined
+Primary account number of sites that
+contain mutiple account numbers(Banks…)</t>
+  </si>
+  <si>
+    <t>*** Needs to be defined</t>
+  </si>
+  <si>
+    <t>Bank Card Type</t>
+  </si>
+  <si>
+    <t>VISA/MasterCard/Discover</t>
+  </si>
+  <si>
+    <t>*** This tie to the combo tables</t>
+  </si>
+  <si>
+    <t>BankCards/?</t>
+  </si>
+  <si>
+    <t>BankCard number</t>
+  </si>
+  <si>
+    <t>Bank  card number</t>
+  </si>
+  <si>
+    <t>BankCard Expiration Date</t>
+  </si>
+  <si>
+    <t>Bank Card Expiration Date</t>
+  </si>
+  <si>
+    <t>BankCards/CVV</t>
+  </si>
+  <si>
+    <t>Bank Card Security Code</t>
+  </si>
+  <si>
+    <t>BankCards/Active</t>
+  </si>
+  <si>
+    <t>Bactive Card Active(Y/N)</t>
+  </si>
+  <si>
+    <t>Is bank card active or not</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -228,15 +351,27 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -259,28 +394,55 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -318,7 +480,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -352,6 +514,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -386,9 +549,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -561,61 +725,61 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:1">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:1">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:1">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:1">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:1">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -626,11 +790,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="42.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.36328125" customWidth="1"/>
+    <col min="5" max="5" width="42.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="36.26953125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -646,8 +817,11 @@
       <c r="E1" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -664,46 +838,49 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>63</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>64</v>
       </c>
       <c r="C3" t="s">
         <v>44</v>
       </c>
       <c r="D3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+        <v>65</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="F3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>72</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="D4" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="E4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
         <v>44</v>
@@ -712,49 +889,55 @@
         <v>46</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
+        <v>48</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="E6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>70</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="D7" t="s">
         <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
+        <v>68</v>
+      </c>
+      <c r="F7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
         <v>44</v>
@@ -763,49 +946,55 @@
         <v>46</v>
       </c>
       <c r="E8" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
+        <v>50</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>80</v>
       </c>
       <c r="D9" t="s">
         <v>46</v>
       </c>
       <c r="E9" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
+        <v>51</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D10" t="s">
         <v>46</v>
       </c>
       <c r="E10" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C11" t="s">
         <v>44</v>
@@ -814,49 +1003,58 @@
         <v>46</v>
       </c>
       <c r="E11" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
+        <v>52</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C12" t="s">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="D12" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="E12" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
+        <v>53</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="D13" t="s">
         <v>46</v>
       </c>
       <c r="E13" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
+        <v>54</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C14" t="s">
         <v>44</v>
@@ -865,15 +1063,18 @@
         <v>46</v>
       </c>
       <c r="E14" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
+        <v>55</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C15" t="s">
         <v>44</v>
@@ -882,15 +1083,18 @@
         <v>46</v>
       </c>
       <c r="E15" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
+        <v>56</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C16" t="s">
         <v>44</v>
@@ -899,24 +1103,172 @@
         <v>46</v>
       </c>
       <c r="E16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
+        <v>57</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="C17" t="s">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="D17" t="s">
         <v>46</v>
       </c>
       <c r="E17" t="s">
-        <v>62</v>
+        <v>58</v>
+      </c>
+      <c r="F17" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" t="s">
+        <v>46</v>
+      </c>
+      <c r="E18" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D19" t="s">
+        <v>46</v>
+      </c>
+      <c r="E19" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" t="s">
+        <v>65</v>
+      </c>
+      <c r="E20" t="s">
+        <v>88</v>
+      </c>
+      <c r="F20" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" t="s">
+        <v>65</v>
+      </c>
+      <c r="E21" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D22" t="s">
+        <v>65</v>
+      </c>
+      <c r="E22" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D23" t="s">
+        <v>65</v>
+      </c>
+      <c r="E23" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" t="s">
+        <v>65</v>
+      </c>
+      <c r="E24" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25" t="s">
+        <v>46</v>
+      </c>
+      <c r="E25" t="s">
+        <v>61</v>
+      </c>
+      <c r="F25" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -925,11 +1277,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -964,82 +1316,82 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:1">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>31</v>
       </c>

</xml_diff>

<commit_message>
Clean up the combo boxes for categories
</commit_message>
<xml_diff>
--- a/MWPV/docs/CategoryItem Layout-gadget.xlsx
+++ b/MWPV/docs/CategoryItem Layout-gadget.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pgmrd\My Drive\MWPV\MWPV\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F34021A8-82C1-449C-98E5-2CF4AA1C13CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C6C1B2-DDE5-42FC-98D0-7E29BE39633F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,12 +17,12 @@
     <sheet name="Fields" sheetId="2" r:id="rId2"/>
     <sheet name="Visibility" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="105">
   <si>
     <t>Category</t>
   </si>
@@ -72,223 +72,207 @@
     <t>Tooltip</t>
   </si>
   <si>
+    <t>Notes</t>
+  </si>
+  <si>
     <t>Title</t>
   </si>
   <si>
+    <t>Text</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Display name for this item</t>
+  </si>
+  <si>
+    <t>CategoryItem/CI_Name</t>
+  </si>
+  <si>
+    <t>Password Name</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Name of this Password entry(app name/web site 
+name/encryupte file or folder name)</t>
+  </si>
+  <si>
+    <t>Can not be modified</t>
+  </si>
+  <si>
+    <t>CategoryItem/CI_Description</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Description of this password entry</t>
+  </si>
+  <si>
+    <t>None Marked optional per review</t>
+  </si>
+  <si>
     <t>Username</t>
   </si>
   <si>
-    <t>Password</t>
-  </si>
-  <si>
-    <t>URL</t>
-  </si>
-  <si>
-    <t>AccountNumber</t>
-  </si>
-  <si>
-    <t>MemberID</t>
-  </si>
-  <si>
-    <t>RoutingNumber</t>
-  </si>
-  <si>
-    <t>Pin</t>
-  </si>
-  <si>
-    <t>RecoveryEmail</t>
-  </si>
-  <si>
-    <t>RecoveryPhone</t>
-  </si>
-  <si>
-    <t>MFAType</t>
-  </si>
-  <si>
-    <t>MFABackupCodes</t>
-  </si>
-  <si>
-    <t>SecurityQuestion</t>
-  </si>
-  <si>
-    <t>SecurityAnswer</t>
-  </si>
-  <si>
-    <t>SupportPhone</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Sign-in URL</t>
-  </si>
-  <si>
-    <t>Account Number</t>
-  </si>
-  <si>
-    <t>Member ID</t>
-  </si>
-  <si>
-    <t>Routing Number</t>
-  </si>
-  <si>
-    <t>PIN</t>
-  </si>
-  <si>
-    <t>Recovery Email</t>
-  </si>
-  <si>
-    <t>Recovery Phone</t>
-  </si>
-  <si>
-    <t>MFA Type</t>
-  </si>
-  <si>
-    <t>MFA Backup Codes</t>
-  </si>
-  <si>
-    <t>Security Question</t>
-  </si>
-  <si>
-    <t>Security Answer</t>
-  </si>
-  <si>
-    <t>Support Phone</t>
-  </si>
-  <si>
-    <t>Text</t>
-  </si>
-  <si>
-    <t>Multiline</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>Display name for this item</t>
-  </si>
-  <si>
     <t>Login username or email</t>
-  </si>
-  <si>
-    <t>Password (masked)</t>
-  </si>
-  <si>
-    <t>Link to sign-in page</t>
-  </si>
-  <si>
-    <t>Bank or account number</t>
-  </si>
-  <si>
-    <t>Membership or policy ID</t>
-  </si>
-  <si>
-    <t>Bank routing number</t>
-  </si>
-  <si>
-    <t>Short numeric PIN</t>
-  </si>
-  <si>
-    <t>Email used for account recovery</t>
-  </si>
-  <si>
-    <t>Phone used for account recovery or MFA</t>
-  </si>
-  <si>
-    <t>e.g., TOTP, SMS, Email, Yubikey</t>
-  </si>
-  <si>
-    <t>One-per-line backup codes</t>
-  </si>
-  <si>
-    <t>Security question prompt</t>
-  </si>
-  <si>
-    <t>Answer to the security question</t>
-  </si>
-  <si>
-    <t>Customer support phone</t>
-  </si>
-  <si>
-    <t>Freeform notes</t>
-  </si>
-  <si>
-    <t>CategoryItem/CI_Name</t>
-  </si>
-  <si>
-    <t>Password Name</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>Can not be modified</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>This is the email recorded for the web site</t>
-  </si>
-  <si>
-    <t>Needs to be added to Category Item Table</t>
-  </si>
-  <si>
-    <t>CateogyryItem/CI_Email</t>
   </si>
   <si>
     <t>Needs to be added to Category Item Table
 Not needed for files/folders and applications</t>
   </si>
   <si>
-    <t>CategoryItem/CI_Description</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Description of this password entry</t>
+    <t>CategoryItemPasswordHistory/CIPaH_Password</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>PasswordBox</t>
+  </si>
+  <si>
+    <t>Password (masked)</t>
+  </si>
+  <si>
+    <t>CategoryItem/CI_Email</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>This is the email recorded for the web site</t>
+  </si>
+  <si>
+    <t>Needs to be added to Category Item Table Ambiguous: consider mapping to CI_RecoveryEmail or adding CI_PrimaryEmail.</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>Sign-in URL</t>
+  </si>
+  <si>
+    <t>Link to sign-in page</t>
   </si>
   <si>
     <t>Needs to be added to Category Item Table
 Required for any website</t>
   </si>
   <si>
-    <t>*** Should we create one json/clob with this
-and the account number in?</t>
-  </si>
-  <si>
-    <t>CategoryItemSecurityQuestions/SecurityQuestion</t>
-  </si>
-  <si>
-    <t>CategoryItemSequerityQuestions/SecurityAnswer</t>
-  </si>
-  <si>
-    <t>*** Not defined yet. Is it needed</t>
-  </si>
-  <si>
-    <t>PasswordBox</t>
-  </si>
-  <si>
-    <t>Multiline/PasswordBox</t>
-  </si>
-  <si>
-    <t>Name of this Password entry(app name/web site 
-name/encryupte file or folder name)</t>
-  </si>
-  <si>
-    <t>*** Is this the user id login?</t>
-  </si>
-  <si>
-    <t>CategoryItemPasswordHistory/CIPaH_Password</t>
+    <t>AccountNumber</t>
+  </si>
+  <si>
+    <t>Account Number</t>
+  </si>
+  <si>
+    <t>TextBox (masked)</t>
+  </si>
+  <si>
+    <t>Bank or account number</t>
   </si>
   <si>
     <t>Needs to be defined
 Primary account number of sites that
-contain mutiple account numbers(Banks…)</t>
-  </si>
-  <si>
-    <t>*** Needs to be defined</t>
+contain mutiple account numbers(Banks…) Changed from PasswordBox to masked TextBox for copy/paste usability.</t>
+  </si>
+  <si>
+    <t>Multiline</t>
+  </si>
+  <si>
+    <t>Freeform notes</t>
+  </si>
+  <si>
+    <t>MemberID</t>
+  </si>
+  <si>
+    <t>Member ID</t>
+  </si>
+  <si>
+    <t>Membership or policy ID</t>
+  </si>
+  <si>
+    <t>RoutingNumber</t>
+  </si>
+  <si>
+    <t>Routing Number</t>
+  </si>
+  <si>
+    <t>Bank routing number</t>
+  </si>
+  <si>
+    <t>Pin</t>
+  </si>
+  <si>
+    <t>PIN</t>
+  </si>
+  <si>
+    <t>Short numeric PIN</t>
+  </si>
+  <si>
+    <t>RecoveryEmail</t>
+  </si>
+  <si>
+    <t>Recovery Email</t>
+  </si>
+  <si>
+    <t>Email used for account recovery</t>
+  </si>
+  <si>
+    <t>*** Not defined yet. Is it needed</t>
+  </si>
+  <si>
+    <t>RecoveryPhone</t>
+  </si>
+  <si>
+    <t>Recovery Phone</t>
+  </si>
+  <si>
+    <t>Phone used for account recovery or MFA</t>
+  </si>
+  <si>
+    <t>MFAType</t>
+  </si>
+  <si>
+    <t>MFA Type</t>
+  </si>
+  <si>
+    <t>e.g., TOTP, SMS, Email, Yubikey</t>
+  </si>
+  <si>
+    <t>MFABackupCodes</t>
+  </si>
+  <si>
+    <t>MFA Backup Codes</t>
+  </si>
+  <si>
+    <t>Multiline/PasswordBox</t>
+  </si>
+  <si>
+    <t>One-per-line backup codes</t>
+  </si>
+  <si>
+    <t>CategoryItemSecurityQuestions/SecurityQuestion</t>
+  </si>
+  <si>
+    <t>Security Question</t>
+  </si>
+  <si>
+    <t>Security question prompt</t>
+  </si>
+  <si>
+    <t>CategoryItemSequerityQuestions/SecurityAnswer</t>
+  </si>
+  <si>
+    <t>Security Answer</t>
+  </si>
+  <si>
+    <t>Answer to the security question</t>
+  </si>
+  <si>
+    <t>BankCards/?</t>
   </si>
   <si>
     <t>Bank Card Type</t>
@@ -300,9 +284,6 @@
     <t>*** This tie to the combo tables</t>
   </si>
   <si>
-    <t>BankCards/?</t>
-  </si>
-  <si>
     <t>BankCard number</t>
   </si>
   <si>
@@ -328,6 +309,39 @@
   </si>
   <si>
     <t>Is bank card active or not</t>
+  </si>
+  <si>
+    <t>SupportPhone</t>
+  </si>
+  <si>
+    <t>Support Phone</t>
+  </si>
+  <si>
+    <t>Customer support phone</t>
+  </si>
+  <si>
+    <t>SecurityQuestion</t>
+  </si>
+  <si>
+    <t>SecurityAnswer</t>
+  </si>
+  <si>
+    <t>Categoryitem/CI_Username</t>
+  </si>
+  <si>
+    <t>CategoryItem/CI_SignInUrl</t>
+  </si>
+  <si>
+    <t>CategoryItem/CI_SecretData</t>
+  </si>
+  <si>
+    <t>CategoryItem/CI_Notes</t>
+  </si>
+  <si>
+    <t>Primary Account Email</t>
+  </si>
+  <si>
+    <t>????????</t>
   </si>
 </sst>
 </file>
@@ -351,27 +365,15 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -394,34 +396,15 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -791,7 +774,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="42.54296875" bestFit="1" customWidth="1"/>
@@ -802,473 +785,472 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>31</v>
+      <c r="F1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="E2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="D3" t="s">
-        <v>65</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>82</v>
+        <v>23</v>
+      </c>
+      <c r="E3" t="s">
+        <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>66</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>65</v>
+        <v>19</v>
       </c>
       <c r="E4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+        <v>28</v>
+      </c>
+      <c r="F4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>99</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="E5" t="s">
-        <v>48</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>71</v>
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>84</v>
+        <v>33</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>80</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="E6" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>100</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="58" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>101</v>
+      </c>
+      <c r="B9" t="s">
         <v>46</v>
       </c>
-      <c r="E7" t="s">
-        <v>68</v>
-      </c>
-      <c r="F7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" t="s">
-        <v>46</v>
-      </c>
-      <c r="E8" t="s">
-        <v>50</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="58" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" t="s">
-        <v>33</v>
-      </c>
       <c r="C9" t="s">
-        <v>80</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>51</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>85</v>
+        <v>48</v>
+      </c>
+      <c r="F9" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>102</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="C10" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D10" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="E10" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="D11" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="E11" t="s">
-        <v>52</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>101</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="C12" t="s">
-        <v>80</v>
+        <v>47</v>
       </c>
       <c r="D12" t="s">
-        <v>65</v>
+        <v>19</v>
       </c>
       <c r="E12" t="s">
-        <v>53</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>101</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C13" t="s">
-        <v>80</v>
+        <v>35</v>
       </c>
       <c r="D13" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="E13" t="s">
-        <v>54</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>86</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>24</v>
+        <v>101</v>
       </c>
       <c r="B14" t="s">
-        <v>37</v>
+        <v>103</v>
       </c>
       <c r="C14" t="s">
-        <v>44</v>
-      </c>
-      <c r="D14" t="s">
-        <v>46</v>
-      </c>
-      <c r="E14" t="s">
-        <v>55</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>79</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>25</v>
+        <v>101</v>
       </c>
       <c r="B15" t="s">
-        <v>38</v>
+        <v>62</v>
       </c>
       <c r="C15" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="E15" t="s">
-        <v>56</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="B16" t="s">
-        <v>39</v>
+        <v>66</v>
       </c>
       <c r="C16" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="D16" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="E16" t="s">
-        <v>57</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>68</v>
       </c>
       <c r="B17" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="C17" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" t="s">
+        <v>70</v>
+      </c>
+      <c r="F17" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" t="s">
+        <v>74</v>
+      </c>
+      <c r="F18" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" t="s">
+        <v>76</v>
+      </c>
+      <c r="C19" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" t="s">
+        <v>73</v>
+      </c>
+      <c r="D20" t="s">
+        <v>19</v>
+      </c>
+      <c r="E20" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>81</v>
       </c>
-      <c r="D17" t="s">
-        <v>46</v>
-      </c>
-      <c r="E17" t="s">
-        <v>58</v>
-      </c>
-      <c r="F17" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D18" t="s">
-        <v>46</v>
-      </c>
-      <c r="E18" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C19" s="4" t="s">
+      <c r="B21" t="s">
+        <v>82</v>
+      </c>
+      <c r="C21" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" t="s">
+        <v>23</v>
+      </c>
+      <c r="E21" t="s">
+        <v>83</v>
+      </c>
+      <c r="F21" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>81</v>
       </c>
-      <c r="D19" t="s">
-        <v>46</v>
-      </c>
-      <c r="E19" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" s="5" t="s">
+      <c r="B22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D22" t="s">
+        <v>23</v>
+      </c>
+      <c r="E22" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>81</v>
+      </c>
+      <c r="B23" t="s">
+        <v>87</v>
+      </c>
+      <c r="C23" t="s">
+        <v>73</v>
+      </c>
+      <c r="D23" t="s">
+        <v>23</v>
+      </c>
+      <c r="E23" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>89</v>
+      </c>
+      <c r="B24" t="s">
         <v>90</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D20" t="s">
-        <v>65</v>
-      </c>
-      <c r="E20" t="s">
-        <v>88</v>
-      </c>
-      <c r="F20" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="5" t="s">
+      <c r="C24" t="s">
+        <v>73</v>
+      </c>
+      <c r="D24" t="s">
+        <v>23</v>
+      </c>
+      <c r="E24" t="s">
         <v>90</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="D21" t="s">
-        <v>65</v>
-      </c>
-      <c r="E21" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="D22" t="s">
-        <v>65</v>
-      </c>
-      <c r="E22" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="D23" t="s">
-        <v>65</v>
-      </c>
-      <c r="E23" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D24" t="s">
-        <v>65</v>
-      </c>
-      <c r="E24" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>30</v>
+        <v>91</v>
       </c>
       <c r="B25" t="s">
-        <v>43</v>
+        <v>92</v>
       </c>
       <c r="C25" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="D25" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="E25" t="s">
-        <v>61</v>
-      </c>
-      <c r="F25" t="s">
-        <v>79</v>
+        <v>93</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>94</v>
+      </c>
+      <c r="B26" t="s">
+        <v>95</v>
+      </c>
+      <c r="C26" t="s">
+        <v>18</v>
+      </c>
+      <c r="D26" t="s">
+        <v>19</v>
+      </c>
+      <c r="E26" t="s">
+        <v>96</v>
+      </c>
+      <c r="F26" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1318,82 +1300,82 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>